<commit_message>
Update TestComplete validation reports - Jenkins build 6
</commit_message>
<xml_diff>
--- a/reports/TestComplete-Validation-Report.xlsx
+++ b/reports/TestComplete-Validation-Report.xlsx
@@ -32,10 +32,10 @@
     <t>Overall Result</t>
   </si>
   <si>
-    <t>5</t>
-  </si>
-  <si>
-    <t>2026-10-08T04:20:24.013Z</t>
+    <t>6</t>
+  </si>
+  <si>
+    <t>2026-10-08T04:37:12.519Z</t>
   </si>
   <si>
     <t>PASS</t>

</xml_diff>